<commit_message>
an error found and fixed in report
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#ELETTRONICASABINAXX/Elettronica_Sabina/Refertos/1.0.0/accreditamento-checklist_V9.0.0.xlsx
+++ b/GATEWAY/A1#111#ELETTRONICASABINAXX/Elettronica_Sabina/Refertos/1.0.0/accreditamento-checklist_V9.0.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\192.168.0.3\xftp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69F04083-DAE6-4426-A602-4006288FF02B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58E3D2C3-1B35-4308-8AFF-72AF2CF0F77C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -285,18 +285,6 @@
 Il Documento CDA2 Referto Specialistica Ambulatoriale dovrà essere composto in modo da risultare valido dal punto di vista sintattico, semantico, terminologico. I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso dalla sezione "CASO DI TEST 25" riportata nei documenti "casi di test RSA" e "CDA2_Referto_Specialistica_Ambulatoriale_OK" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
   </si>
   <si>
-    <t>Viene richiamato il servizio di validazione "https://&lt;HOST&gt;:&lt;PORT&gt;/v&lt;major&gt;/documents/validation" al fine di testare la gestione degli errori terminologici sui Dati (status code 400), secondo quanto descritto in https://github.com/ministero-salute/it-fse-support/tree/main/doc/integrazione-gateway. 
-I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 26" riportata nei documenti "casi di test RSA" e "CDA2_Referto_Specialistica_Ambulatoriale_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
-  </si>
-  <si>
-    <t>Viene richiamato il servizio di validazione "https://&lt;HOST&gt;:&lt;PORT&gt;/v&lt;major&gt;/documents/validation" al fine di testare la gestione degli errori sintattici sui Dati (status code 400), secondo quanto descritto in https://github.com/ministero-salute/it-fse-support/tree/main/doc/integrazione-gateway.
-I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 27" riportata nei documenti "casi di test RSA" e "CDA2_Referto_Specialistica_Ambulatoriale_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
-  </si>
-  <si>
-    <t>Viene richiamato il servizio di validazione "https://&lt;HOST&gt;:&lt;PORT&gt;/v&lt;major&gt;/documents/validation" al fine di testare la gestione degli errori terminologici sui Dati (status code 400), secondo quanto descritto in https://github.com/ministero-salute/it-fse-support/tree/main/doc/integrazione-gateway. 
-I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 28" riportata nei documenti "casi di test RSA" e "CDA2_Referto_Specialistica_Ambulatoriale_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
-  </si>
-  <si>
     <t>Razionale di Applicabilità</t>
   </si>
   <si>
@@ -437,6 +425,18 @@
   </si>
   <si>
     <t>Si</t>
+  </si>
+  <si>
+    <t>Viene richiamato il servizio di validazione "https://&lt;HOST&gt;:&lt;PORT&gt;/v&lt;major&gt;/documents/validation", al fine di una futura pubblicazione, con esito positivo (status code 201), secondo quanto descritto in https://github.com/ministero-salute/it-fse-support/tree/main/doc/integrazione-gateway.
+I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 26" riportata nei documenti "casi di test RSA" e "CDA2_Referto_Specialistica_Ambulatoriale_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
+  </si>
+  <si>
+    <t>Viene richiamato il servizio di validazione "https://&lt;HOST&gt;:&lt;PORT&gt;/v&lt;major&gt;/documents/validation", al fine di una futura pubblicazione, con esito positivo (status code 201), secondo quanto descritto in https://github.com/ministero-salute/it-fse-support/tree/main/doc/integrazione-gateway.
+I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 27" riportata nei documenti "casi di test RSA" e "CDA2_Referto_Specialistica_Ambulatoriale_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
+  </si>
+  <si>
+    <t>Viene richiamato il servizio di validazione "https://&lt;HOST&gt;:&lt;PORT&gt;/v&lt;major&gt;/documents/validation", al fine di una futura pubblicazione, con esito positivo (status code 201), secondo quanto descritto in https://github.com/ministero-salute/it-fse-support/tree/main/doc/integrazione-gateway.
+I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 28" riportata nei documenti "casi di test RSA" e "CDA2_Referto_Specialistica_Ambulatoriale_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
   </si>
 </sst>
 </file>
@@ -1020,6 +1020,21 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1041,21 +1056,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1384,7 +1384,7 @@
     </row>
     <row r="4" spans="1:1" ht="85.5" x14ac:dyDescent="0.45">
       <c r="A4" s="33" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="270.75" x14ac:dyDescent="0.45">
@@ -2538,12 +2538,12 @@
       <c r="W1" s="9"/>
     </row>
     <row r="2" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="40" t="s">
+      <c r="A2" s="45" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="41"/>
-      <c r="C2" s="42"/>
-      <c r="D2" s="41"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="46"/>
       <c r="F2" s="6"/>
       <c r="G2" s="6"/>
       <c r="H2" s="6"/>
@@ -2564,14 +2564,14 @@
       <c r="W2" s="9"/>
     </row>
     <row r="3" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="43" t="s">
+      <c r="A3" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="44"/>
-      <c r="C3" s="49" t="s">
-        <v>70</v>
-      </c>
-      <c r="D3" s="41"/>
+      <c r="B3" s="49"/>
+      <c r="C3" s="54" t="s">
+        <v>67</v>
+      </c>
+      <c r="D3" s="46"/>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
       <c r="H3" s="6"/>
@@ -2592,12 +2592,12 @@
       <c r="W3" s="9"/>
     </row>
     <row r="4" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A4" s="45"/>
-      <c r="B4" s="46"/>
-      <c r="C4" s="49" t="s">
-        <v>71</v>
-      </c>
-      <c r="D4" s="41"/>
+      <c r="A4" s="50"/>
+      <c r="B4" s="51"/>
+      <c r="C4" s="54" t="s">
+        <v>68</v>
+      </c>
+      <c r="D4" s="46"/>
       <c r="E4" s="4"/>
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
@@ -2619,12 +2619,12 @@
       <c r="W4" s="9"/>
     </row>
     <row r="5" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="47"/>
-      <c r="B5" s="48"/>
-      <c r="C5" s="49" t="s">
-        <v>72</v>
-      </c>
-      <c r="D5" s="41"/>
+      <c r="A5" s="52"/>
+      <c r="B5" s="53"/>
+      <c r="C5" s="54" t="s">
+        <v>69</v>
+      </c>
+      <c r="D5" s="46"/>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
@@ -2645,8 +2645,8 @@
       <c r="W5" s="9"/>
     </row>
     <row r="6" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A6" s="38"/>
-      <c r="B6" s="39"/>
+      <c r="A6" s="43"/>
+      <c r="B6" s="44"/>
       <c r="C6" s="10"/>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
@@ -2791,26 +2791,26 @@
       <c r="C10" s="31" t="s">
         <v>44</v>
       </c>
-      <c r="D10" s="50" t="s">
-        <v>73</v>
+      <c r="D10" s="38" t="s">
+        <v>70</v>
       </c>
       <c r="E10" s="32" t="s">
         <v>46</v>
       </c>
-      <c r="F10" s="51">
+      <c r="F10" s="39">
         <v>46119</v>
       </c>
-      <c r="G10" s="52" t="s">
-        <v>79</v>
-      </c>
-      <c r="H10" s="52" t="s">
-        <v>85</v>
-      </c>
-      <c r="I10" s="53" t="s">
-        <v>86</v>
-      </c>
-      <c r="J10" s="54" t="s">
-        <v>97</v>
+      <c r="G10" s="40" t="s">
+        <v>76</v>
+      </c>
+      <c r="H10" s="40" t="s">
+        <v>82</v>
+      </c>
+      <c r="I10" s="41" t="s">
+        <v>83</v>
+      </c>
+      <c r="J10" s="42" t="s">
+        <v>94</v>
       </c>
       <c r="K10" s="28"/>
       <c r="L10" s="28"/>
@@ -2838,26 +2838,26 @@
       <c r="C11" s="31" t="s">
         <v>44</v>
       </c>
-      <c r="D11" s="50" t="s">
-        <v>74</v>
+      <c r="D11" s="38" t="s">
+        <v>71</v>
       </c>
       <c r="E11" s="32" t="s">
         <v>47</v>
       </c>
-      <c r="F11" s="51">
+      <c r="F11" s="39">
         <v>46119</v>
       </c>
-      <c r="G11" s="52" t="s">
-        <v>80</v>
-      </c>
-      <c r="H11" s="52" t="s">
-        <v>87</v>
-      </c>
-      <c r="I11" s="53" t="s">
-        <v>88</v>
-      </c>
-      <c r="J11" s="54" t="s">
-        <v>97</v>
+      <c r="G11" s="40" t="s">
+        <v>77</v>
+      </c>
+      <c r="H11" s="40" t="s">
+        <v>84</v>
+      </c>
+      <c r="I11" s="41" t="s">
+        <v>85</v>
+      </c>
+      <c r="J11" s="42" t="s">
+        <v>94</v>
       </c>
       <c r="K11" s="28"/>
       <c r="L11" s="28"/>
@@ -2885,26 +2885,26 @@
       <c r="C12" s="31" t="s">
         <v>44</v>
       </c>
-      <c r="D12" s="50" t="s">
-        <v>75</v>
+      <c r="D12" s="38" t="s">
+        <v>72</v>
       </c>
       <c r="E12" s="32" t="s">
-        <v>48</v>
-      </c>
-      <c r="F12" s="51">
+        <v>95</v>
+      </c>
+      <c r="F12" s="39">
         <v>46119</v>
       </c>
-      <c r="G12" s="52" t="s">
-        <v>81</v>
-      </c>
-      <c r="H12" s="52" t="s">
-        <v>89</v>
-      </c>
-      <c r="I12" s="53" t="s">
-        <v>90</v>
-      </c>
-      <c r="J12" s="54" t="s">
-        <v>97</v>
+      <c r="G12" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="H12" s="40" t="s">
+        <v>86</v>
+      </c>
+      <c r="I12" s="41" t="s">
+        <v>87</v>
+      </c>
+      <c r="J12" s="42" t="s">
+        <v>94</v>
       </c>
       <c r="K12" s="28"/>
       <c r="L12" s="27"/>
@@ -2932,26 +2932,26 @@
       <c r="C13" s="31" t="s">
         <v>44</v>
       </c>
-      <c r="D13" s="50" t="s">
-        <v>76</v>
+      <c r="D13" s="38" t="s">
+        <v>73</v>
       </c>
       <c r="E13" s="32" t="s">
-        <v>49</v>
-      </c>
-      <c r="F13" s="51">
+        <v>96</v>
+      </c>
+      <c r="F13" s="39">
         <v>46119</v>
       </c>
-      <c r="G13" s="52" t="s">
-        <v>82</v>
-      </c>
-      <c r="H13" s="52" t="s">
-        <v>91</v>
-      </c>
-      <c r="I13" s="53" t="s">
-        <v>92</v>
-      </c>
-      <c r="J13" s="54" t="s">
-        <v>97</v>
+      <c r="G13" s="40" t="s">
+        <v>79</v>
+      </c>
+      <c r="H13" s="40" t="s">
+        <v>88</v>
+      </c>
+      <c r="I13" s="41" t="s">
+        <v>89</v>
+      </c>
+      <c r="J13" s="42" t="s">
+        <v>94</v>
       </c>
       <c r="K13" s="28"/>
       <c r="L13" s="27"/>
@@ -2979,26 +2979,26 @@
       <c r="C14" s="31" t="s">
         <v>44</v>
       </c>
-      <c r="D14" s="50" t="s">
-        <v>77</v>
+      <c r="D14" s="38" t="s">
+        <v>74</v>
       </c>
       <c r="E14" s="32" t="s">
-        <v>50</v>
-      </c>
-      <c r="F14" s="51">
+        <v>97</v>
+      </c>
+      <c r="F14" s="39">
         <v>46119</v>
       </c>
-      <c r="G14" s="52" t="s">
-        <v>83</v>
-      </c>
-      <c r="H14" s="52" t="s">
-        <v>93</v>
-      </c>
-      <c r="I14" s="53" t="s">
+      <c r="G14" s="40" t="s">
+        <v>80</v>
+      </c>
+      <c r="H14" s="40" t="s">
+        <v>90</v>
+      </c>
+      <c r="I14" s="41" t="s">
+        <v>91</v>
+      </c>
+      <c r="J14" s="42" t="s">
         <v>94</v>
-      </c>
-      <c r="J14" s="54" t="s">
-        <v>97</v>
       </c>
       <c r="K14" s="28"/>
       <c r="L14" s="28"/>
@@ -3026,26 +3026,26 @@
       <c r="C15" s="31" t="s">
         <v>44</v>
       </c>
-      <c r="D15" s="50" t="s">
-        <v>78</v>
+      <c r="D15" s="38" t="s">
+        <v>75</v>
       </c>
       <c r="E15" s="32" t="s">
-        <v>50</v>
-      </c>
-      <c r="F15" s="51">
+        <v>97</v>
+      </c>
+      <c r="F15" s="39">
         <v>46119</v>
       </c>
-      <c r="G15" s="52" t="s">
-        <v>84</v>
-      </c>
-      <c r="H15" s="52" t="s">
-        <v>95</v>
-      </c>
-      <c r="I15" s="53" t="s">
-        <v>96</v>
-      </c>
-      <c r="J15" s="54" t="s">
-        <v>97</v>
+      <c r="G15" s="40" t="s">
+        <v>81</v>
+      </c>
+      <c r="H15" s="40" t="s">
+        <v>92</v>
+      </c>
+      <c r="I15" s="41" t="s">
+        <v>93</v>
+      </c>
+      <c r="J15" s="42" t="s">
+        <v>94</v>
       </c>
       <c r="K15" s="28"/>
       <c r="L15" s="28"/>
@@ -5268,42 +5268,42 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -5327,22 +5327,22 @@
   <sheetData>
     <row r="1" spans="1:7" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A1" s="26" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B1" s="11" t="s">
         <v>20</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D1" s="36" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="G1" s="34" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="14.25" x14ac:dyDescent="0.45">
@@ -5350,10 +5350,10 @@
         <v>44</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C2" s="35" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D2" s="37"/>
     </row>
@@ -6327,7 +6327,7 @@
     </row>
     <row r="2" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="4" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>45</v>
@@ -6335,10 +6335,10 @@
     </row>
     <row r="3" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="4" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -7352,15 +7352,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A92AB09DCDF6014AA0D6826BF29E2C8E" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="58b13f75919cba2dcad85f84b1d5db00">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1e76d14e-d0ce-457c-8343-9b55836d9ead" xmlns:ns3="a56712a3-8dfd-4688-917a-22f0cf513b89" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a3b16ea44285e6579c272a3325f660d0" ns2:_="" ns3:_="">
     <xsd:import namespace="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
@@ -7624,6 +7615,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -7637,14 +7637,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1AD72871-87C6-44C4-AEDE-C35BE2C233EE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7659,6 +7651,14 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>